<commit_message>
Atualização para o Gemini 3.1 Flash e refactoring do codigo
</commit_message>
<xml_diff>
--- a/destinatarios/destinatarios.xlsx
+++ b/destinatarios/destinatarios.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t xml:space="preserve">Destinatários</t>
   </si>
@@ -31,34 +31,10 @@
     <t xml:space="preserve">Mensagem</t>
   </si>
   <si>
-    <t xml:space="preserve">COPED_ESUMP_GO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crie o parecer pedagógico do evento: &lt;NOME_EVENTO&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COEVE_ESUMP_GO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crie o Projeto de Evento de &lt;NOME_EVENTO&gt; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">COEDI_ESUMP_GO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crie a arte gráfica para o evento: &lt;NOME_EVENTO&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">COTEC_ESUMP_GO</t>
   </si>
   <si>
     <t xml:space="preserve">Crie as páginas Moodle e a inscrição para: &lt;NOME_EVENTO&gt; </t>
-  </si>
-  <si>
-    <t xml:space="preserve">COCOM_ESUMP_GO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Crie a divulgação pertinente para o evento: &lt;NOME_EVENTO&gt;</t>
   </si>
 </sst>
 </file>
@@ -149,16 +125,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -298,7 +278,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.76"/>
@@ -322,37 +302,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:B5"/>

</xml_diff>